<commit_message>
docs : Sua lai BOM V0.1
</commit_message>
<xml_diff>
--- a/hardware/bom/BOM_V0.1.xlsx
+++ b/hardware/bom/BOM_V0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DOWNLOAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C39FBA-7ECE-456E-BEB5-636B6AD933B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC363D8B-3923-44A8-B624-3EBD6788EF66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="65">
   <si>
     <t>STT</t>
   </si>
@@ -57,24 +57,12 @@
     <t>SL</t>
   </si>
   <si>
-    <t>Đơn giá (VND)</t>
-  </si>
-  <si>
-    <t>Thành tiền (VND)</t>
-  </si>
-  <si>
     <t>Trạng thái duyệt</t>
   </si>
   <si>
     <t>PPG AFE</t>
   </si>
   <si>
-    <t>Module MAX30101 breakout (I2C, LED đỏ/xanh lá/IR tích hợp)</t>
-  </si>
-  <si>
-    <t>MAX30102 module có pad chọn 3V3 (chỉ đỏ+IR); ProtoCentral AFE4490 breakout (SPI, đỏ+IR)</t>
-  </si>
-  <si>
     <t>Bắt buộc</t>
   </si>
   <si>
@@ -96,18 +84,6 @@
     <t>Tùy chọn</t>
   </si>
   <si>
-    <t>Nguồn</t>
-  </si>
-  <si>
-    <t>Nguồn sạch 3,3 V cho các board AFE (LDO nhiễu thấp hoặc nguồn bàn của phòng lab)</t>
-  </si>
-  <si>
-    <t>Cấp qua USB nếu board có LDO riêng</t>
-  </si>
-  <si>
-    <t>Khuyến nghị</t>
-  </si>
-  <si>
     <t>Kết nối</t>
   </si>
   <si>
@@ -225,9 +201,6 @@
     <t>3M Red Dot 2560</t>
   </si>
   <si>
-    <t>Dây jumper</t>
-  </si>
-  <si>
     <t>__</t>
   </si>
   <si>
@@ -237,20 +210,35 @@
     <t>Điện cực ECG (dry electrode)</t>
   </si>
   <si>
-    <t xml:space="preserve">TỔNG </t>
-  </si>
-  <si>
     <t>BIOPAC ELDRY-SP-FLAT</t>
+  </si>
+  <si>
+    <t>Dây chuyên dụng breadboard</t>
+  </si>
+  <si>
+    <t>1 (hộp)</t>
+  </si>
+  <si>
+    <t>BIOPAC ELDRY-SP-DOME</t>
+  </si>
+  <si>
+    <t>MAX30001 là ECG AFE chuyên dụng, phù hợp mục tiêu thu ECG chất lượng và kiểm chứng AFE trước khi thiết kế phần cứng riêng</t>
+  </si>
+  <si>
+    <t>Có giao tiếp SPI/I²C, đủ để kết nối các AFE/cảm biến và thuận tiện lập trình, debug qua USB</t>
+  </si>
+  <si>
+    <t>Dễ mua, phù hợp với dự án ở tiến độ hiện tại</t>
+  </si>
+  <si>
+    <t>Phù hợp với hướng phát triển dạng đeo tay của dự án</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
-  </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -284,18 +272,12 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
       <sz val="13"/>
       <name val="Arial"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -306,12 +288,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
         <bgColor rgb="FF333333"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -342,10 +318,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -355,18 +330,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -632,320 +596,246 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
-    <col min="4" max="4" width="34" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="6" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="4" max="5" width="34" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="6" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="4">
+        <v>1</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="4">
+        <v>1</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="4">
+        <v>1</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="4">
+        <v>2</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="C8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="4">
+        <v>2</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="4">
+        <v>3</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="4">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="3" t="s">
+      <c r="H10" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="4">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="s">
+      <c r="G11" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="5">
-        <v>2</v>
-      </c>
-      <c r="G4" s="6"/>
-      <c r="H4" s="7" t="str">
-        <f t="shared" ref="H4:H12" si="0">IF(G4="","",F4*G4)</f>
-        <v/>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="4">
-        <v>2</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="5">
-        <v>1</v>
-      </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="4">
-        <v>3</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="5">
-        <v>1</v>
-      </c>
-      <c r="G6" s="8"/>
-      <c r="H6" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="4">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="5">
-        <v>1</v>
-      </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="4">
-        <v>5</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="5">
-        <v>1</v>
-      </c>
-      <c r="G8" s="6"/>
-      <c r="H8" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
-        <v>7</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" s="5">
-        <v>1</v>
-      </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="4">
-        <v>8</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="5">
-        <v>2</v>
-      </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="4">
-        <v>9</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="5">
-        <v>2</v>
-      </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="4">
-        <v>10</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="5">
-        <v>1</v>
-      </c>
-      <c r="G12" s="6"/>
-      <c r="H12" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="G13" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="H13" s="10">
-        <f>SUM(H4:H12)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="I4:I12" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="H4:H11" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"CHỜ DUYỆT,ĐÃ DUYỆT,TỪ CHỐI,ĐÃ ĐẶT,ĐÃ NHẬN"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -966,127 +856,127 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C6" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="4"/>
-    </row>
-    <row r="6" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="4" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="4"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="4"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="C11" s="3"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C13" s="3"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="4"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="4"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="4"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
docs : Sua lai BOM V0.1 (#11)
</commit_message>
<xml_diff>
--- a/hardware/bom/BOM_V0.1.xlsx
+++ b/hardware/bom/BOM_V0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DOWNLOAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C39FBA-7ECE-456E-BEB5-636B6AD933B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC363D8B-3923-44A8-B624-3EBD6788EF66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="65">
   <si>
     <t>STT</t>
   </si>
@@ -57,24 +57,12 @@
     <t>SL</t>
   </si>
   <si>
-    <t>Đơn giá (VND)</t>
-  </si>
-  <si>
-    <t>Thành tiền (VND)</t>
-  </si>
-  <si>
     <t>Trạng thái duyệt</t>
   </si>
   <si>
     <t>PPG AFE</t>
   </si>
   <si>
-    <t>Module MAX30101 breakout (I2C, LED đỏ/xanh lá/IR tích hợp)</t>
-  </si>
-  <si>
-    <t>MAX30102 module có pad chọn 3V3 (chỉ đỏ+IR); ProtoCentral AFE4490 breakout (SPI, đỏ+IR)</t>
-  </si>
-  <si>
     <t>Bắt buộc</t>
   </si>
   <si>
@@ -96,18 +84,6 @@
     <t>Tùy chọn</t>
   </si>
   <si>
-    <t>Nguồn</t>
-  </si>
-  <si>
-    <t>Nguồn sạch 3,3 V cho các board AFE (LDO nhiễu thấp hoặc nguồn bàn của phòng lab)</t>
-  </si>
-  <si>
-    <t>Cấp qua USB nếu board có LDO riêng</t>
-  </si>
-  <si>
-    <t>Khuyến nghị</t>
-  </si>
-  <si>
     <t>Kết nối</t>
   </si>
   <si>
@@ -225,9 +201,6 @@
     <t>3M Red Dot 2560</t>
   </si>
   <si>
-    <t>Dây jumper</t>
-  </si>
-  <si>
     <t>__</t>
   </si>
   <si>
@@ -237,20 +210,35 @@
     <t>Điện cực ECG (dry electrode)</t>
   </si>
   <si>
-    <t xml:space="preserve">TỔNG </t>
-  </si>
-  <si>
     <t>BIOPAC ELDRY-SP-FLAT</t>
+  </si>
+  <si>
+    <t>Dây chuyên dụng breadboard</t>
+  </si>
+  <si>
+    <t>1 (hộp)</t>
+  </si>
+  <si>
+    <t>BIOPAC ELDRY-SP-DOME</t>
+  </si>
+  <si>
+    <t>MAX30001 là ECG AFE chuyên dụng, phù hợp mục tiêu thu ECG chất lượng và kiểm chứng AFE trước khi thiết kế phần cứng riêng</t>
+  </si>
+  <si>
+    <t>Có giao tiếp SPI/I²C, đủ để kết nối các AFE/cảm biến và thuận tiện lập trình, debug qua USB</t>
+  </si>
+  <si>
+    <t>Dễ mua, phù hợp với dự án ở tiến độ hiện tại</t>
+  </si>
+  <si>
+    <t>Phù hợp với hướng phát triển dạng đeo tay của dự án</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
-  </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -284,18 +272,12 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
       <sz val="13"/>
       <name val="Arial"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -306,12 +288,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
         <bgColor rgb="FF333333"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -342,10 +318,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -355,18 +330,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -632,320 +596,246 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
-    <col min="4" max="4" width="34" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="6" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="4" max="5" width="34" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="6" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="4">
+        <v>1</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="4">
+        <v>1</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="4">
+        <v>1</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="4">
+        <v>2</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="C8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="4">
+        <v>2</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="4">
+        <v>3</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="4">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="3" t="s">
+      <c r="H10" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="4">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="s">
+      <c r="G11" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="5">
-        <v>2</v>
-      </c>
-      <c r="G4" s="6"/>
-      <c r="H4" s="7" t="str">
-        <f t="shared" ref="H4:H12" si="0">IF(G4="","",F4*G4)</f>
-        <v/>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="4">
-        <v>2</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="5">
-        <v>1</v>
-      </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="4">
-        <v>3</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="5">
-        <v>1</v>
-      </c>
-      <c r="G6" s="8"/>
-      <c r="H6" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="4">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="5">
-        <v>1</v>
-      </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="4">
-        <v>5</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="5">
-        <v>1</v>
-      </c>
-      <c r="G8" s="6"/>
-      <c r="H8" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
-        <v>7</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" s="5">
-        <v>1</v>
-      </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="4">
-        <v>8</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="5">
-        <v>2</v>
-      </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="4">
-        <v>9</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="5">
-        <v>2</v>
-      </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="4">
-        <v>10</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="5">
-        <v>1</v>
-      </c>
-      <c r="G12" s="6"/>
-      <c r="H12" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="G13" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="H13" s="10">
-        <f>SUM(H4:H12)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="I4:I12" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="H4:H11" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"CHỜ DUYỆT,ĐÃ DUYỆT,TỪ CHỐI,ĐÃ ĐẶT,ĐÃ NHẬN"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -966,127 +856,127 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C6" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="4"/>
-    </row>
-    <row r="6" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="4" t="s">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="4"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="4"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="C11" s="3"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C13" s="3"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="4"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="4"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="4"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>